<commit_message>
feat(finance): real ordered-to-shipped split + the full arithmetic walk
All-Orders report replaces the guessed gap: 4,459 ordered in Aug -> 120
cancelled (2.7%, the REAL rate, not the 15.5% the old proxy implied) - 1
pending - 3 unfulfillable - 204 not shipped by month end = 4,131 shipped,
which reconciles to the 4,133 Amazon paid on within 2 units of cross-month
timing. The old proxy compared a Sun-Sat week grid (2 Aug-5 Sep) against a
calendar month.

Section 7 now shows HOW THE TOTAL IS BUILT — every component from sales
through GST, refunds, fee givebacks, fees, promos, EMI, reimbursements, TCS
and TDS, footing to the settlement, then to contribution, then after ads. The
bottom line can be followed line by line instead of appearing from nowhere.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nner8RaGyk95YsJkMTo8Tg
</commit_message>
<xml_diff>
--- a/data/processed/reconciliation_NEXLEV_2026-08.xlsx
+++ b/data/processed/reconciliation_NEXLEV_2026-08.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,219 +469,219 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4892</v>
+        <v>4459</v>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>on Amazon, 3P</t>
+          <t>orders placed this month</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Units Amazon shipped and paid on</t>
+          <t xml:space="preserve">  of which cancelled</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4133</v>
+        <v>-120</v>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>the financial basis</t>
+          <t>the real cancellation rate</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Product sales - GST NOT included</t>
+          <t xml:space="preserve">  of which not shipped by month end</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11621287.74</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
+        <v>-204</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>our revenue; every % below is against this</t>
+          <t>ships next month - timing, not lost</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GST collected from customers</t>
+          <t xml:space="preserve">  Units Amazon shipped and paid on</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2062051.32</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>17.7%</t>
-        </is>
-      </c>
+        <v>4133</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>held in trust - never ours</t>
+          <t>the financial basis</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  What customers actually paid</t>
+          <t xml:space="preserve">  Product sales - GST NOT included</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>13683339.06</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
+        <v>11621287.74</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>sales + GST = the money that came in</t>
+          <t>our revenue; every % below is against this</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GST collected from customers</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2062051.32</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>17.7%</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>held in trust - never ours</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>WHAT CAME BACK</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
+          <t xml:space="preserve">  What customers actually paid</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>13683339.06</v>
+      </c>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>sales + GST = the money that came in</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Units refunded</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>567</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>13.7%</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>of units shipped</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sale value refunded</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>-1753159.5</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>15.1%</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>of sales</t>
-        </is>
-      </c>
+          <t>WHAT CAME BACK</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Fees Amazon gave back on those refunds</t>
+          <t xml:space="preserve">  Units refunded</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>106869.05</v>
-      </c>
-      <c r="C12" t="inlineStr"/>
+        <v>567</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>13.7%</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>commission + closing returned; FBA fee never is</t>
+          <t>of units shipped</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sale value refunded</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>-1753159.5</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>15.1%</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>of sales</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>WHAT AMAZON DEDUCTED (before GST on fees)</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
+          <t xml:space="preserve">  Fees Amazon gave back on those refunds</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>106869.05</v>
+      </c>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>commission + closing returned; FBA fee never is</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Commission (referral)</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>-826239.8100000001</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>7.1%</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FBA fulfilment (pick, pack, deliver)</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>-596204.52</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>5.1%</t>
-        </is>
-      </c>
+          <t>WHAT AMAZON DEDUCTED (before GST on fees)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Closing fee</t>
+          <t xml:space="preserve">  Commission (referral)</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-177166</v>
+        <v>-826239.8100000001</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1.5%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -689,15 +689,15 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Storage</t>
+          <t xml:space="preserve">  FBA fulfilment (pick, pack, deliver)</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-111891.38</v>
+        <v>-596204.52</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.0%</t>
+          <t>5.1%</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -705,146 +705,152 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Long-term storage (aged stock)</t>
+          <t xml:space="preserve">  Closing fee</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-18510.93</v>
+        <v>-177166</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.2%</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>stock sitting too long</t>
-        </is>
-      </c>
+          <t>1.5%</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Removals and other service fees</t>
+          <t xml:space="preserve">  Storage</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-15105.44</v>
-      </c>
-      <c r="C20" t="inlineStr"/>
+        <v>-111891.38</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1.0%</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  TOTAL AMAZON FEES</t>
+          <t xml:space="preserve">  Long-term storage (aged stock)</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-1711657.45</v>
+        <v>-18510.93</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>0.2%</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>of sales, before GST on fees</t>
+          <t>stock sitting too long</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Removals and other service fees</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>-15105.44</v>
+      </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>WHAT WE PAID FOR OURSELVES</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
+          <t xml:space="preserve">  TOTAL AMAZON FEES</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>-1711657.45</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>of sales, before GST on fees</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Coupons and promotions</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>-153674.29</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1.3%</t>
-        </is>
-      </c>
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  No-cost EMI / bank offers</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>-69514.82000000001</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>0.6%</t>
-        </is>
-      </c>
+          <t>WHAT WE PAID FOR OURSELVES</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Advertising</t>
+          <t xml:space="preserve">  Coupons and promotions</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>-1501598.67</v>
+        <v>-153674.29</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>12.9%</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>billed separately, not in settlement</t>
-        </is>
-      </c>
+          <t>1.3%</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  No-cost EMI / bank offers</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>-69514.82000000001</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>0.6%</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>WHAT AMAZON PAID BACK</t>
+          <t xml:space="preserve">  Advertising</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>210889.26</v>
+        <v>-1501598.67</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1.8%</t>
+          <t>12.9%</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>reimbursements for lost/damaged stock, fee corrections</t>
+          <t>billed separately, not in settlement</t>
         </is>
       </c>
     </row>
@@ -857,194 +863,220 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TAX HELD BACK (not a cost - you get it back)</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
+          <t>WHAT AMAZON PAID BACK</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>210889.26</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1.8%</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>reimbursements for lost/damaged stock, fee corrections</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  TCS at 0.5% of net sales</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>-49015.15</v>
-      </c>
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>goes to your GST cash ledger - ACCEPT IT MONTHLY on the portal</t>
-        </is>
-      </c>
+      <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">  TDS at 0.1% of gross sales</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>-11592.94</v>
-      </c>
+          <t>TAX HELD BACK (not a cost - you get it back)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>claim in your income tax return</t>
-        </is>
-      </c>
+      <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
-      <c r="B33" t="inlineStr"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TCS at 0.5% of net sales</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>-49015.15</v>
+      </c>
       <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>goes to your GST cash ledger - ACCEPT IT MONTHLY on the portal</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>THE BOTTOM LINE</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr"/>
+          <t xml:space="preserve">  TDS at 0.1% of gross sales</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>-11592.94</v>
+      </c>
       <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>claim in your income tax return</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Amazon should pay us</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>9707251.27</v>
-      </c>
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>cash, including the GST we must pass on</t>
-        </is>
-      </c>
+      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  less GST we owe the government</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>-2011026.85</v>
-      </c>
+          <t>THE BOTTOM LINE</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>output GST less refunds, less credit on fee GST, less TCS</t>
-        </is>
-      </c>
+      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  CONTRIBUTION BEFORE COST OF GOODS</t>
+          <t xml:space="preserve">  Amazon should pay us</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>7696224.42</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>66.2%</t>
-        </is>
-      </c>
+        <v>9707251.27</v>
+      </c>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>of sales</t>
+          <t>cash, including the GST we must pass on</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  After advertising</t>
+          <t xml:space="preserve">  less GST we owe the government</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>6194625.75</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>53.3%</t>
-        </is>
-      </c>
+        <v>-2011026.85</v>
+      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>STILL NOT PROFIT - cost of goods not included</t>
+          <t>output GST less refunds, less credit on fee GST, less TCS</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CONTRIBUTION BEFORE COST OF GOODS</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>7696224.42</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>66.2%</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>of sales</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>PROOF THIS IS COMPLETE</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
+          <t xml:space="preserve">  After advertising</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>6194625.75</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>53.3%</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>STILL NOT PROFIT - cost of goods not included</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Event types Amazon reported</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>6</v>
-      </c>
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>every one classified above</t>
-        </is>
-      </c>
+      <c r="D41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Event types that were empty</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>27</v>
-      </c>
+          <t>PROOF THIS IS COMPLETE</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>nothing ignored</t>
-        </is>
-      </c>
+      <c r="D42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Settlement cycles tied to Amazon's own totals</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>12 of 12</t>
-        </is>
+          <t xml:space="preserve">  Event types Amazon reported</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>6</v>
       </c>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
+        <is>
+          <t>every one classified above</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Event types that were empty</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>27</v>
+      </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>nothing ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Settlement cycles tied to Amazon's own totals</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>12 of 12</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
         <is>
           <t>each cycle matches to the paisa</t>
         </is>
@@ -1061,7 +1093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1094,15 +1126,15 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Units ordered (weekly report, order-date basis)</t>
+          <t>Units ordered in the month</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4892</v>
+        <v>4459</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>different date basis from shipped</t>
+          <t>All-Orders report, order date</t>
         </is>
       </c>
     </row>
@@ -1114,15 +1146,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Units shipped (what Amazon paid on)</t>
+          <t xml:space="preserve">  less cancelled</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4133</v>
+        <v>-120</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>financial basis</t>
+          <t>2.7% of orders - the REAL cancellation rate</t>
         </is>
       </c>
     </row>
@@ -1134,17 +1166,13 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ordered but not shipped</t>
+          <t xml:space="preserve">  less pending (payment not authorised)</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>759</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>NOT all cancellations - month-end timing + pending orders; needs All-Orders report to split</t>
-        </is>
-      </c>
+        <v>-1</v>
+      </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1154,17 +1182,13 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Product sales (GST NOT included)</t>
+          <t xml:space="preserve">  less unfulfillable</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>11621287.74</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>P&amp;L revenue</t>
-        </is>
-      </c>
+        <v>-3</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1174,85 +1198,88 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Shipping and gift wrap collected</t>
+          <t xml:space="preserve">  less not shipped by month end</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>66766.37</v>
-      </c>
-      <c r="D6" t="inlineStr"/>
+        <v>-204</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ships next month</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2. RETURNS</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Units refunded</t>
-        </is>
+          <t>1. SALES</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f> Shipped from this month's orders</f>
+        <v/>
       </c>
       <c r="C7" t="n">
-        <v>567</v>
+        <v>4131</v>
       </c>
       <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2. RETURNS</t>
+          <t>1. SALES</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Return rate % (in-month, mixed cohorts)</t>
+          <t>Units shipped (what Amazon paid on)</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>13.72</v>
+        <v>4133</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>these refunds mostly belong to earlier months' shipments</t>
+          <t>financial basis; differs from 4131 by cross-month timing</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2. RETURNS</t>
+          <t>1. SALES</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Sale value refunded (GST NOT included)</t>
+          <t>Product sales (GST NOT included)</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-1753159.5</v>
-      </c>
-      <c r="D9" t="inlineStr"/>
+        <v>11621287.74</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>P&amp;L revenue</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2. RETURNS</t>
+          <t>1. SALES</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Commission on refunds (ex-GST)</t>
+          <t>Shipping and gift wrap collected</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>125100.29</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>given back to us</t>
-        </is>
-      </c>
+        <v>66766.37</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1262,17 +1289,13 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FixedClosingFee on refunds (ex-GST)</t>
+          <t>Units refunded</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>12623</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>given back to us</t>
-        </is>
-      </c>
+        <v>567</v>
+      </c>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1282,15 +1305,15 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>GiftwrapChargeback on refunds (ex-GST)</t>
+          <t>Return rate % (in-month, mixed cohorts)</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>25.42</v>
+        <v>13.72</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>given back to us</t>
+          <t>these refunds mostly belong to earlier months' shipments</t>
         </is>
       </c>
     </row>
@@ -1302,17 +1325,13 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RefundCommission on refunds (ex-GST)</t>
+          <t>Sale value refunded (GST NOT included)</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-31750</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Amazon kept this</t>
-        </is>
-      </c>
+        <v>-1753159.5</v>
+      </c>
+      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1322,11 +1341,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ShippingChargeback on refunds (ex-GST)</t>
+          <t>Commission on refunds (ex-GST)</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>870.34</v>
+        <v>125100.29</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1337,66 +1356,82 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>3. AMAZON FEES (ex-GST)</t>
+          <t>2. RETURNS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Commission (referral)</t>
+          <t>FixedClosingFee on refunds (ex-GST)</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-826239.8100000001</v>
-      </c>
-      <c r="D15" t="inlineStr"/>
+        <v>12623</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>given back to us</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3. AMAZON FEES (ex-GST)</t>
+          <t>2. RETURNS</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>FBA fulfilment</t>
+          <t>GiftwrapChargeback on refunds (ex-GST)</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-596204.52</v>
-      </c>
-      <c r="D16" t="inlineStr"/>
+        <v>25.42</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>given back to us</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3. AMAZON FEES (ex-GST)</t>
+          <t>2. RETURNS</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Closing fee</t>
+          <t>RefundCommission on refunds (ex-GST)</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-177166</v>
-      </c>
-      <c r="D17" t="inlineStr"/>
+        <v>-31750</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Amazon kept this</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3. AMAZON FEES (ex-GST)</t>
+          <t>2. RETURNS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Other selling fees</t>
+          <t>ShippingChargeback on refunds (ex-GST)</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>-4586.44</v>
-      </c>
-      <c r="D18" t="inlineStr"/>
+        <v>870.34</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>given back to us</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1406,17 +1441,13 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FBAStorageFee</t>
+          <t>Commission (referral)</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>-111891.38</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>FBA Inventory Storage Fee</t>
-        </is>
-      </c>
+        <v>-826239.8100000001</v>
+      </c>
+      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1426,17 +1457,13 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FBALongTermStorageFee</t>
+          <t>FBA fulfilment</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>-18510.93</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>FBA Long Term Storage Fee</t>
-        </is>
-      </c>
+        <v>-596204.52</v>
+      </c>
+      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1446,17 +1473,13 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FBARemovalFee</t>
+          <t>Closing fee</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>-9320</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>FBA Removal Order: Return Fee</t>
-        </is>
-      </c>
+        <v>-177166</v>
+      </c>
+      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1466,17 +1489,13 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>MFNPostageFee</t>
+          <t>Other selling fees</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>-1199</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>ServiceFee</t>
-        </is>
-      </c>
+        <v>-4586.44</v>
+      </c>
+      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1486,15 +1505,15 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>TechnologyFee</t>
+          <t>FBAStorageFee</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>-111891.38</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>RefusedDelivery</t>
+          <t>FBA Inventory Storage Fee</t>
         </is>
       </c>
     </row>
@@ -1506,15 +1525,15 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>TechnologyFee</t>
+          <t>FBALongTermStorageFee</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>-18510.93</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ShippingAddressUndeliverable</t>
+          <t>FBA Long Term Storage Fee</t>
         </is>
       </c>
     </row>
@@ -1526,15 +1545,15 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>TechnologyFee</t>
+          <t>FBARemovalFee</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>-9320</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>UnableToDeliver</t>
+          <t>FBA Removal Order: Return Fee</t>
         </is>
       </c>
     </row>
@@ -1546,11 +1565,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Subscription</t>
+          <t>MFNPostageFee</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>-1199</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1566,15 +1585,15 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>FBAPerUnitFulfillmentFee</t>
+          <t>TechnologyFee</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>204.36</v>
+        <v>0</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>UnableToDeliver</t>
+          <t>RefusedDelivery</t>
         </is>
       </c>
     </row>
@@ -1586,15 +1605,15 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>FBAWeightBasedFee</t>
+          <t>TechnologyFee</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1001</v>
+        <v>0</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>UnableToDeliver</t>
+          <t>ShippingAddressUndeliverable</t>
         </is>
       </c>
     </row>
@@ -1606,15 +1625,15 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>FBAPerUnitFulfillmentFee</t>
+          <t>TechnologyFee</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1639.65</v>
+        <v>0</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ShippingAddressUndeliverable</t>
+          <t>UnableToDeliver</t>
         </is>
       </c>
     </row>
@@ -1626,15 +1645,15 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>FBAPerUnitFulfillmentFee</t>
+          <t>Subscription</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>4343.62</v>
+        <v>0</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>RefusedDelivery</t>
+          <t>ServiceFee</t>
         </is>
       </c>
     </row>
@@ -1646,15 +1665,15 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>FBAWeightBasedFee</t>
+          <t>FBAPerUnitFulfillmentFee</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>7577</v>
+        <v>204.36</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>ShippingAddressUndeliverable</t>
+          <t>UnableToDeliver</t>
         </is>
       </c>
     </row>
@@ -1670,143 +1689,143 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>18695</v>
+        <v>1001</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>RefusedDelivery</t>
+          <t>UnableToDeliver</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>4. WE FUNDED</t>
+          <t>3. AMAZON FEES (ex-GST)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Coupons / promotions</t>
+          <t>FBAPerUnitFulfillmentFee</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>-153674.29</v>
-      </c>
-      <c r="D33" t="inlineStr"/>
+        <v>1639.65</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>ShippingAddressUndeliverable</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>4. WE FUNDED</t>
+          <t>3. AMAZON FEES (ex-GST)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>No-cost EMI / bank offers</t>
+          <t>FBAPerUnitFulfillmentFee</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>-69514.82000000001</v>
-      </c>
-      <c r="D34" t="inlineStr"/>
+        <v>4343.62</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>RefusedDelivery</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>4. WE FUNDED</t>
+          <t>3. AMAZON FEES (ex-GST)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Advertising (from our AMS data)</t>
+          <t>FBAWeightBasedFee</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>-1501598.67</v>
+        <v>7577</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>billed outside settlement - CONFIRM if GST-inclusive</t>
+          <t>ShippingAddressUndeliverable</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>5. CREDITS</t>
+          <t>3. AMAZON FEES (ex-GST)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Reversal Reimbursement</t>
+          <t>FBAWeightBasedFee</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>101864.35</v>
+        <v>18695</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>compensation - no GST</t>
+          <t>RefusedDelivery</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>5. CREDITS</t>
+          <t>4. WE FUNDED</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Free Replacement Refund Items</t>
+          <t>Coupons / promotions</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>42851.01</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>compensation - no GST</t>
-        </is>
-      </c>
+        <v>-153674.29</v>
+      </c>
+      <c r="D37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>5. CREDITS</t>
+          <t>4. WE FUNDED</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Lostordamagedreimbursement</t>
+          <t>No-cost EMI / bank offers</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1114.52</v>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>compensation - no GST</t>
-        </is>
-      </c>
+        <v>-69514.82000000001</v>
+      </c>
+      <c r="D38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5. CREDITS</t>
+          <t>4. WE FUNDED</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Warehouse Damage</t>
+          <t>Advertising (from our AMS data)</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1821.61</v>
+        <v>-1501598.67</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>compensation - no GST</t>
+          <t>billed outside settlement - CONFIRM if GST-inclusive</t>
         </is>
       </c>
     </row>
@@ -1818,15 +1837,15 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Commissioncorrection</t>
+          <t>Reversal Reimbursement</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>65468.13</v>
+        <v>101864.35</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>fee credit - carries GST, reverses ITC</t>
+          <t>compensation - no GST</t>
         </is>
       </c>
     </row>
@@ -1838,11 +1857,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Payment Retraction Items</t>
+          <t>Free Replacement Refund Items</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>-2230.36</v>
+        <v>42851.01</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1853,76 +1872,80 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>6. GST AND TAX (not profit)</t>
+          <t>5. CREDITS</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Output GST collected from customers</t>
+          <t>Lostordamagedreimbursement</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2062051.32</v>
+        <v>1114.52</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>held in trust - never ours</t>
+          <t>compensation - no GST</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>6. GST AND TAX (not profit)</t>
+          <t>5. CREDITS</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Output GST reversed on refunds</t>
+          <t>Warehouse Damage</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>-310107.66</v>
-      </c>
-      <c r="D43" t="inlineStr"/>
+        <v>1821.61</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>compensation - no GST</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>6. GST AND TAX (not profit)</t>
+          <t>5. CREDITS</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ITC on Amazon fees (reclaimable)</t>
+          <t>Commissioncorrection</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>308098.34</v>
+        <v>65468.13</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>tie to Amazon's tax invoice AND GSTR-2B</t>
+          <t>fee credit - carries GST, reverses ITC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>6. GST AND TAX (not profit)</t>
+          <t>5. CREDITS</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>TCS withheld u/s 52 (0.5% of net sales)</t>
+          <t>Payment Retraction Items</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>-49015.15</v>
+        <v>-2230.36</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>PREPAYMENT ASSET - accept monthly in the GST portal or it is stranded</t>
+          <t>compensation - no GST</t>
         </is>
       </c>
     </row>
@@ -1934,15 +1957,15 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>TDS withheld u/s 194-O (0.1% of gross)</t>
+          <t>Output GST collected from customers</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>-11592.94</v>
+        <v>2062051.32</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>RECOVERABLE in ITR - charged on gross, so returns are a permanent drag</t>
+          <t>held in trust - never ours</t>
         </is>
       </c>
     </row>
@@ -1954,121 +1977,429 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Net GST still to remit in cash</t>
+          <t>Output GST reversed on refunds</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>-2011026.85</v>
+        <v>-310107.66</v>
       </c>
       <c r="D47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>7. BOTTOM LINE</t>
+          <t>6. GST AND TAX (not profit)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Amazon should settle (cash basis, GST-inclusive)</t>
+          <t>ITC on Amazon fees (reclaimable)</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>9707251.27</v>
+        <v>308098.34</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>compare with deposits - cycles straddle the month end</t>
+          <t>tie to Amazon's tax invoice AND GSTR-2B</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>7. BOTTOM LINE</t>
+          <t>6. GST AND TAX (not profit)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>less: net GST to remit to government</t>
+          <t>TCS withheld u/s 52 (0.5% of net sales)</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>-2011026.85</v>
-      </c>
-      <c r="D49" t="inlineStr"/>
+        <v>-49015.15</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>PREPAYMENT ASSET - accept monthly in the GST portal or it is stranded</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>7. BOTTOM LINE</t>
+          <t>6. GST AND TAX (not profit)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Marketplace contribution BEFORE COGS</t>
+          <t>TDS withheld u/s 194-O (0.1% of gross)</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>7696224.42</v>
-      </c>
-      <c r="D50" t="inlineStr"/>
+        <v>-11592.94</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>RECOVERABLE in ITR - charged on gross, so returns are a permanent drag</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>7. BOTTOM LINE</t>
+          <t>6. GST AND TAX (not profit)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>After advertising, BEFORE COGS</t>
+          <t>Net GST still to remit in cash</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>6194625.75</v>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>NOT profit - landed cost of goods is not in this file</t>
-        </is>
-      </c>
+        <v>-2011026.85</v>
+      </c>
+      <c r="D51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>9. COMPLETENESS</t>
+          <t>7. HOW THE TOTAL IS BUILT</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Event lists Amazon returned with data</t>
+          <t>Product sales (GST not included)</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>6</v>
+        <v>11621287.74</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>AdjustmentEventList, AffordabilityExpenseEventList, AffordabilityExpenseReversalEventList, RefundEventList, ServiceFeeEventList, ShipmentEventList</t>
+          <t>what we sold</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>9. COMPLETENESS</t>
+          <t>7. HOW THE TOTAL IS BUILT</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
+          <t>plus GST collected from customers</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>2062051.32</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>comes in with the sale, goes out to the government</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>7. HOW THE TOTAL IS BUILT</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>plus shipping and gift wrap</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>66766.37</v>
+      </c>
+      <c r="D54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>7. HOW THE TOTAL IS BUILT</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>less refunds to customers</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>-2076295.91</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>sale value + GST returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>7. HOW THE TOTAL IS BUILT</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>plus fees Amazon returned on refunds</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>126105.48</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>commission and closing come back; FBA fee does not</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>7. HOW THE TOTAL IS BUILT</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>less Amazon fees (including GST on fees)</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>-2019755.79</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>commission, FBA, closing, storage, removals</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>7. HOW THE TOTAL IS BUILT</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>less coupons and promotions</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>-153674.29</v>
+      </c>
+      <c r="D58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>7. HOW THE TOTAL IS BUILT</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>less no-cost EMI and bank offers</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>-69514.82000000001</v>
+      </c>
+      <c r="D59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>7. HOW THE TOTAL IS BUILT</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>plus reimbursements and corrections</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>210889.26</v>
+      </c>
+      <c r="D60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>7. HOW THE TOTAL IS BUILT</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>less TCS withheld</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>-49015.15</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>you reclaim this in GST</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>7. HOW THE TOTAL IS BUILT</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>less TDS withheld</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>-11592.94</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>you reclaim this in your ITR</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>8. BOTTOM LINE</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>AMAZON SHOULD PAY US</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>9707251.27</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>add up everything above - this is the settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>8. BOTTOM LINE</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>less GST we owe the government</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>-2011026.85</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>output GST, less GST refunded, less credit on fee GST, less TCS already withheld</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>8. BOTTOM LINE</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>MARKETPLACE CONTRIBUTION BEFORE COGS</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>7696224.42</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>what the marketplace actually left us</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>8. BOTTOM LINE</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>less advertising</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>-1501598.67</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>billed separately by Amazon Ads, never in the settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>8. BOTTOM LINE</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>AFTER ADVERTISING, BEFORE COGS</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>6194625.75</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>NOT profit - the landed cost of the goods still has to come off</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>10. COMPLETENESS</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Event lists Amazon returned with data</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>6</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>AdjustmentEventList, AffordabilityExpenseEventList, AffordabilityExpenseReversalEventList, RefundEventList, ServiceFeeEventList, ShipmentEventList</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>10. COMPLETENESS</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
           <t>Event lists returned EMPTY</t>
         </is>
       </c>
-      <c r="C53" t="n">
+      <c r="C69" t="n">
         <v>27</v>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D69" t="inlineStr">
         <is>
           <t>incl. ShipmentSettleEventList - must stay empty or revenue double-counts</t>
         </is>

</xml_diff>